<commit_message>
generate new output files
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_PER_loopback_tutorial/Rev02/BOM/BOM_UZ_PER_loopback_tutorial_[No Variations]_Rev02.xlsx
+++ b/Project Outputs for UZ_PER_loopback_tutorial/Rev02/BOM/BOM_UZ_PER_loopback_tutorial_[No Variations]_Rev02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johan\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{199FC8B5-92EE-42A1-9EA1-97E6BE1E7BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5082AA8E-112C-449A-9186-E44CC0AAF35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{772E28E0-5732-4BD7-952F-F9D4E0A9517A}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4F12F980-6CBB-4C00-A7D7-F8132859CDFE}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UZ_PER_loopback_tutorial_ N" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="59">
   <si>
     <t>Designator</t>
   </si>
@@ -197,10 +197,10 @@
     <t>X2</t>
   </si>
   <si>
-    <t>30 Position, Classic PCB Header Strips, 0.100&amp;quot; pitch</t>
-  </si>
-  <si>
-    <t>TSW-115-07-G-D</t>
+    <t>2x15 Pins</t>
+  </si>
+  <si>
+    <t>200-TSW11507GD</t>
   </si>
   <si>
     <t>TSW-115-XX-YY-D</t>
@@ -611,7 +611,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E509B4CD-60AC-4B2D-980C-2BDAC77E07D4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D211519-B064-40A9-811E-023EEA06DC87}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -837,10 +837,12 @@
       <c r="B8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="1"/>
+      <c r="C8" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D8" s="1"/>
       <c r="E8" s="2" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>54</v>
@@ -848,7 +850,9 @@
       <c r="G8" s="1">
         <v>1</v>
       </c>
-      <c r="H8" s="1"/>
+      <c r="H8" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>

</xml_diff>

<commit_message>
replace resistors and LEDs
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_PER_loopback_tutorial/Rev02/BOM/BOM_UZ_PER_loopback_tutorial_[No Variations]_Rev02.xlsx
+++ b/Project Outputs for UZ_PER_loopback_tutorial/Rev02/BOM/BOM_UZ_PER_loopback_tutorial_[No Variations]_Rev02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johan\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5082AA8E-112C-449A-9186-E44CC0AAF35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{133567D5-129B-4B6B-8959-7DF2C7F506B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4F12F980-6CBB-4C00-A7D7-F8132859CDFE}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{362819B9-CF51-4E4B-8819-E77123F198CE}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UZ_PER_loopback_tutorial_ N" sheetId="1" r:id="rId1"/>
@@ -131,7 +131,7 @@
     <t>SMD resistor 0.1%, SMD resistor 0.1%, 10ppm, SMD resistor 1%, SMD resistor E24 series</t>
   </si>
   <si>
-    <t>66-PCFW0603LF031001B, 279-RQ73C1J10KBTD, 71-CRCW0603-24.9K-E3 , 660-RK73B1JTTD222J, 660-RK73B1JTTD432J</t>
+    <t>66-PCFW0603LF031001B, 279-RQ73C1J10KBTD, 71-CRCW0603-24.9K-E3 , 660-RK73B1JTTD103J, 660-RK73B1JTTD432J</t>
   </si>
   <si>
     <t>[NoValue], =LCSC Part Number</t>
@@ -143,7 +143,7 @@
     <t>[NoValue], LCSC</t>
   </si>
   <si>
-    <t>1k, 10k, 24k9, 2k2, 4k3</t>
+    <t>1k, 10k, 24k9, 4k3</t>
   </si>
   <si>
     <t>Serial1</t>
@@ -611,7 +611,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D211519-B064-40A9-811E-023EEA06DC87}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD44101-3D92-4E30-83E4-D166DB9CA6FF}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>